<commit_message>
added more materials to the BOM
</commit_message>
<xml_diff>
--- a/variations/Camden/V0.2.1/BOM-SPARC-Camden-V0.2.1.xlsx
+++ b/variations/Camden/V0.2.1/BOM-SPARC-Camden-V0.2.1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\github\Smart-Pack-for-Advanced-Research-and-Control\variations\Camden\V0.2.1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/34105aa9bb97034c/Documents/GitHub/Smart-Pack-for-Advanced-Research-and-Control/variations/Camden/V0.2.1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AB63AE7-4EA2-4048-A932-9087CFBE3B31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{7AB63AE7-4EA2-4048-A932-9087CFBE3B31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{618831F3-FDE0-4B0A-89D1-ACC6546CD8FB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="bill_of_materials" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="154">
   <si>
     <t>Total Cost</t>
   </si>
@@ -480,6 +480,24 @@
   </si>
   <si>
     <t>pack of 50, need 2</t>
+  </si>
+  <si>
+    <t>contact nut</t>
+  </si>
+  <si>
+    <t>contact washer</t>
+  </si>
+  <si>
+    <t>https://www.grainger.com/product/Flat-Washer-18-8-26WC34</t>
+  </si>
+  <si>
+    <t>https://www.grainger.com/product/Hex-Nut-Std-Hex-22YK33</t>
+  </si>
+  <si>
+    <t>Flat Washer: 18-8, Stainless Steel, M6 Screw Sz, 6.62 mm In Dia, 12 mm Out Dia, 18-8, 50 PK</t>
+  </si>
+  <si>
+    <t>Hex Nut: Std Hex, M6x1.00 Thread, 10 mm Hex Wd, 5 mm Hex Ht, Stainless Steel, 18-8, Plain, 50 PK</t>
   </si>
 </sst>
 </file>
@@ -489,7 +507,7 @@
   <numFmts count="1">
     <numFmt numFmtId="7" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -504,6 +522,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -527,7 +558,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -550,6 +581,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -887,22 +924,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
   <dimension ref="A1:L48"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="74" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="12.28515625" customWidth="1"/>
-    <col min="7" max="7" width="69.42578125" customWidth="1"/>
+    <col min="3" max="3" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="12.26953125" customWidth="1"/>
+    <col min="7" max="7" width="69.453125" customWidth="1"/>
     <col min="8" max="8" width="76" customWidth="1"/>
-    <col min="9" max="9" width="83.5703125" customWidth="1"/>
-    <col min="10" max="10" width="62.5703125" customWidth="1"/>
-    <col min="11" max="11" width="55.85546875" customWidth="1"/>
+    <col min="9" max="9" width="83.54296875" customWidth="1"/>
+    <col min="10" max="10" width="62.54296875" customWidth="1"/>
+    <col min="11" max="11" width="55.81640625" customWidth="1"/>
     <col min="12" max="12" width="51" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -940,7 +977,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -964,7 +1001,7 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>102</v>
       </c>
@@ -987,7 +1024,7 @@
       </c>
       <c r="H3" s="4"/>
     </row>
-    <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -1011,7 +1048,7 @@
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
     </row>
-    <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -1037,7 +1074,7 @@
       </c>
       <c r="I5" s="2"/>
     </row>
-    <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -1063,7 +1100,7 @@
       </c>
       <c r="I6" s="3"/>
     </row>
-    <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>29</v>
       </c>
@@ -1089,7 +1126,7 @@
       </c>
       <c r="I7" s="2"/>
     </row>
-    <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>26</v>
       </c>
@@ -1111,7 +1148,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>68</v>
       </c>
@@ -1135,7 +1172,7 @@
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
     </row>
-    <row r="10" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>33</v>
       </c>
@@ -1159,7 +1196,7 @@
       <c r="H10" s="3"/>
       <c r="I10" s="5"/>
     </row>
-    <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>36</v>
       </c>
@@ -1182,7 +1219,7 @@
       </c>
       <c r="H11" s="5"/>
     </row>
-    <row r="12" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>37</v>
       </c>
@@ -1205,7 +1242,7 @@
       </c>
       <c r="H12" s="5"/>
     </row>
-    <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>43</v>
       </c>
@@ -1227,7 +1264,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>45</v>
       </c>
@@ -1254,7 +1291,7 @@
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
     </row>
-    <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>49</v>
       </c>
@@ -1277,7 +1314,7 @@
       </c>
       <c r="H15" s="5"/>
     </row>
-    <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>52</v>
       </c>
@@ -1300,7 +1337,7 @@
       </c>
       <c r="H16" s="5"/>
     </row>
-    <row r="17" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>123</v>
       </c>
@@ -1323,7 +1360,7 @@
       </c>
       <c r="H17" s="5"/>
     </row>
-    <row r="18" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>111</v>
       </c>
@@ -1346,7 +1383,7 @@
       </c>
       <c r="H18" s="3"/>
     </row>
-    <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>55</v>
       </c>
@@ -1369,7 +1406,7 @@
       </c>
       <c r="H19" s="5"/>
     </row>
-    <row r="20" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>112</v>
       </c>
@@ -1392,7 +1429,7 @@
       </c>
       <c r="H20" s="5"/>
     </row>
-    <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>58</v>
       </c>
@@ -1415,7 +1452,7 @@
       </c>
       <c r="H21" s="5"/>
     </row>
-    <row r="22" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>61</v>
       </c>
@@ -1438,7 +1475,7 @@
       </c>
       <c r="H22" s="5"/>
     </row>
-    <row r="23" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>64</v>
       </c>
@@ -1461,7 +1498,7 @@
       </c>
       <c r="H23" s="5"/>
     </row>
-    <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>67</v>
       </c>
@@ -1484,7 +1521,7 @@
       </c>
       <c r="H24" s="5"/>
     </row>
-    <row r="25" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>110</v>
       </c>
@@ -1507,7 +1544,7 @@
       </c>
       <c r="H25" s="5"/>
     </row>
-    <row r="26" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>75</v>
       </c>
@@ -1532,7 +1569,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>77</v>
       </c>
@@ -1555,7 +1592,7 @@
       </c>
       <c r="H27" s="5"/>
     </row>
-    <row r="28" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>79</v>
       </c>
@@ -1578,7 +1615,7 @@
       </c>
       <c r="H28" s="5"/>
     </row>
-    <row r="29" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>84</v>
       </c>
@@ -1601,7 +1638,7 @@
       </c>
       <c r="H29" s="5"/>
     </row>
-    <row r="30" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>86</v>
       </c>
@@ -1626,7 +1663,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>89</v>
       </c>
@@ -1649,7 +1686,7 @@
       </c>
       <c r="H31" s="5"/>
     </row>
-    <row r="32" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>90</v>
       </c>
@@ -1673,7 +1710,7 @@
       <c r="H32" s="3"/>
       <c r="I32" s="5"/>
     </row>
-    <row r="33" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>117</v>
       </c>
@@ -1695,7 +1732,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>97</v>
       </c>
@@ -1718,7 +1755,7 @@
       </c>
       <c r="H34" s="5"/>
     </row>
-    <row r="35" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>106</v>
       </c>
@@ -1741,7 +1778,7 @@
       </c>
       <c r="H35" s="5"/>
     </row>
-    <row r="36" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>108</v>
       </c>
@@ -1764,7 +1801,7 @@
       </c>
       <c r="H36" s="5"/>
     </row>
-    <row r="37" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>116</v>
       </c>
@@ -1786,7 +1823,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>125</v>
       </c>
@@ -1808,7 +1845,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>128</v>
       </c>
@@ -1830,7 +1867,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>133</v>
       </c>
@@ -1854,7 +1891,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>137</v>
       </c>
@@ -1874,7 +1911,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>139</v>
       </c>
@@ -1900,7 +1937,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>144</v>
       </c>
@@ -1924,27 +1961,55 @@
       </c>
       <c r="H43" s="1"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="7"/>
-      <c r="E44" s="6"/>
-      <c r="F44" s="6"/>
-      <c r="G44" s="1"/>
+    <row r="44" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B44" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="C44" s="2">
+        <v>1</v>
+      </c>
+      <c r="D44" s="7">
+        <v>2.73</v>
+      </c>
+      <c r="E44" s="6">
+        <v>2.73</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>151</v>
+      </c>
       <c r="H44" s="1"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="7"/>
-      <c r="E45" s="6"/>
-      <c r="F45" s="6"/>
-      <c r="G45" s="1"/>
+    <row r="45" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="C45" s="2">
+        <v>1</v>
+      </c>
+      <c r="D45" s="7">
+        <v>1.2</v>
+      </c>
+      <c r="E45" s="6">
+        <v>1.2</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>150</v>
+      </c>
       <c r="H45" s="1"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -1954,7 +2019,7 @@
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -1964,7 +2029,7 @@
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="D48" s="7" t="s">
         <v>24</v>
       </c>

</xml_diff>

<commit_message>
added materials to BOM
</commit_message>
<xml_diff>
--- a/variations/Camden/V0.2.1/BOM-SPARC-Camden-V0.2.1.xlsx
+++ b/variations/Camden/V0.2.1/BOM-SPARC-Camden-V0.2.1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/34105aa9bb97034c/Documents/GitHub/Smart-Pack-for-Advanced-Research-and-Control/variations/Camden/V0.2.1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{7AB63AE7-4EA2-4048-A932-9087CFBE3B31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{618831F3-FDE0-4B0A-89D1-ACC6546CD8FB}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="13_ncr:1_{7AB63AE7-4EA2-4048-A932-9087CFBE3B31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7AD4F2C-7ACD-4A9B-BDD8-87D87ED80A4A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="160">
   <si>
     <t>Total Cost</t>
   </si>
@@ -498,6 +498,24 @@
   </si>
   <si>
     <t>Hex Nut: Std Hex, M6x1.00 Thread, 10 mm Hex Wd, 5 mm Hex Ht, Stainless Steel, 18-8, Plain, 50 PK</t>
+  </si>
+  <si>
+    <t>22 gauge red wire</t>
+  </si>
+  <si>
+    <t>22 gauge black wire</t>
+  </si>
+  <si>
+    <t>APPROVED VENDOR Automotive Wire: TXL, 100 ft, 1 Conductor, 22 AWG, Black, 60 V Volt</t>
+  </si>
+  <si>
+    <t>https://www.grainger.com/product/Automotive-Wire-TXL-862FY9</t>
+  </si>
+  <si>
+    <t>APPROVED VENDOR Automotive Wire: TXL, 100 ft, 1 Conductor, 22 AWG, Red, 60 V Volt</t>
+  </si>
+  <si>
+    <t>https://www.grainger.com/product/Automotive-Wire-TXL-862FZ5</t>
   </si>
 </sst>
 </file>
@@ -507,7 +525,7 @@
   <numFmts count="1">
     <numFmt numFmtId="7" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -529,6 +547,18 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -558,7 +588,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -588,6 +618,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -604,6 +640,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -923,7 +963,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
@@ -1015,7 +1055,7 @@
         <v>9.99</v>
       </c>
       <c r="E3" s="6">
-        <f t="shared" ref="E3:E40" si="0">C3*D3</f>
+        <f t="shared" ref="E3:E42" si="0">C3*D3</f>
         <v>9.99</v>
       </c>
       <c r="F3" s="6"/>
@@ -1150,892 +1190,933 @@
     </row>
     <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>69</v>
+        <v>155</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>156</v>
       </c>
       <c r="C9" s="2">
         <v>1</v>
       </c>
       <c r="D9" s="6">
-        <v>90.99</v>
+        <v>10.72</v>
       </c>
       <c r="E9" s="6">
         <f t="shared" si="0"/>
-        <v>90.99</v>
+        <v>10.72</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
+        <v>157</v>
+      </c>
     </row>
     <row r="10" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" s="2">
-        <v>1</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="C10" s="2"/>
       <c r="D10" s="6">
-        <v>162.72</v>
+        <v>10.72</v>
       </c>
       <c r="E10" s="6">
-        <f t="shared" si="0"/>
-        <v>162.72</v>
+        <v>10.72</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="H10" s="3"/>
-      <c r="I10" s="5"/>
+        <v>159</v>
+      </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="C11" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" s="6">
-        <v>23.08</v>
+        <v>90.99</v>
       </c>
       <c r="E11" s="6">
         <f t="shared" si="0"/>
-        <v>46.16</v>
+        <v>90.99</v>
       </c>
       <c r="F11" s="6"/>
       <c r="G11" s="3" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
     </row>
     <row r="12" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>39</v>
+        <v>33</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="C12" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" s="6">
-        <v>7.26</v>
+        <v>162.72</v>
       </c>
       <c r="E12" s="6">
         <f t="shared" si="0"/>
-        <v>14.52</v>
+        <v>162.72</v>
       </c>
       <c r="F12" s="6"/>
       <c r="G12" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="H12" s="5"/>
+        <v>35</v>
+      </c>
+      <c r="H12" s="3"/>
+      <c r="I12" s="5"/>
     </row>
     <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C13" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" s="6">
-        <v>8.98</v>
+        <v>23.08</v>
       </c>
       <c r="E13" s="6">
         <f t="shared" si="0"/>
-        <v>8.98</v>
+        <v>46.16</v>
       </c>
       <c r="F13" s="6"/>
       <c r="G13" s="3" t="s">
-        <v>42</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="H13" s="5"/>
     </row>
     <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>46</v>
+        <v>37</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="C14" s="2">
         <v>2</v>
       </c>
       <c r="D14" s="6">
-        <v>74.89</v>
+        <v>7.26</v>
       </c>
       <c r="E14" s="6">
         <f t="shared" si="0"/>
-        <v>149.78</v>
+        <v>14.52</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
+        <v>41</v>
+      </c>
+      <c r="H14" s="5"/>
     </row>
     <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C15" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" s="6">
-        <v>10.17</v>
+        <v>8.98</v>
       </c>
       <c r="E15" s="6">
-        <f>C15*D15</f>
-        <v>20.34</v>
+        <f t="shared" si="0"/>
+        <v>8.98</v>
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="H15" s="5"/>
+        <v>42</v>
+      </c>
     </row>
     <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C16" s="2">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D16" s="6">
-        <v>1.77</v>
+        <v>74.89</v>
       </c>
       <c r="E16" s="6">
         <f t="shared" si="0"/>
-        <v>14.16</v>
+        <v>149.78</v>
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="H16" s="5"/>
-    </row>
-    <row r="17" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+    </row>
+    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>123</v>
+        <v>49</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>122</v>
+        <v>48</v>
       </c>
       <c r="C17" s="2">
         <v>2</v>
       </c>
       <c r="D17" s="6">
-        <v>23.66</v>
+        <v>10.17</v>
       </c>
       <c r="E17" s="6">
-        <f t="shared" si="0"/>
-        <v>47.32</v>
+        <f>C17*D17</f>
+        <v>20.34</v>
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="3" t="s">
-        <v>124</v>
+        <v>50</v>
       </c>
       <c r="H17" s="5"/>
     </row>
-    <row r="18" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>111</v>
+        <v>52</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C18" s="2">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D18" s="6">
-        <v>15.02</v>
+        <v>1.77</v>
       </c>
       <c r="E18" s="6">
         <f t="shared" si="0"/>
-        <v>15.02</v>
+        <v>14.16</v>
       </c>
       <c r="F18" s="6"/>
       <c r="G18" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="H18" s="3"/>
-    </row>
-    <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>115</v>
+      </c>
+      <c r="H18" s="5"/>
+    </row>
+    <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>55</v>
+        <v>123</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C19" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" s="6">
-        <v>12.46</v>
+        <v>23.66</v>
       </c>
       <c r="E19" s="6">
         <f t="shared" si="0"/>
-        <v>12.46</v>
+        <v>47.32</v>
       </c>
       <c r="F19" s="6"/>
       <c r="G19" s="3" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="H19" s="5"/>
     </row>
-    <row r="20" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C20" s="2">
         <v>1</v>
       </c>
       <c r="D20" s="6">
-        <v>15.13</v>
+        <v>15.02</v>
       </c>
       <c r="E20" s="6">
         <f t="shared" si="0"/>
-        <v>15.13</v>
+        <v>15.02</v>
       </c>
       <c r="F20" s="6"/>
       <c r="G20" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="H20" s="5"/>
-    </row>
-    <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+      <c r="H20" s="3"/>
+    </row>
+    <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>59</v>
+        <v>114</v>
       </c>
       <c r="C21" s="2">
         <v>1</v>
       </c>
       <c r="D21" s="6">
-        <v>29.3</v>
+        <v>12.46</v>
       </c>
       <c r="E21" s="6">
         <f t="shared" si="0"/>
-        <v>29.3</v>
+        <v>12.46</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="3" t="s">
-        <v>60</v>
+        <v>113</v>
       </c>
       <c r="H21" s="5"/>
     </row>
-    <row r="22" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>61</v>
+        <v>112</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C22" s="2">
         <v>1</v>
       </c>
       <c r="D22" s="6">
-        <v>4.09</v>
+        <v>15.13</v>
       </c>
       <c r="E22" s="6">
         <f t="shared" si="0"/>
-        <v>4.09</v>
+        <v>15.13</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="3" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="H22" s="5"/>
     </row>
-    <row r="23" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C23" s="2">
         <v>1</v>
       </c>
       <c r="D23" s="6">
-        <v>147.52000000000001</v>
+        <v>29.3</v>
       </c>
       <c r="E23" s="6">
         <f t="shared" si="0"/>
-        <v>147.52000000000001</v>
+        <v>29.3</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="3" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H23" s="5"/>
     </row>
-    <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="C24" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D24" s="6">
-        <v>1.45</v>
+        <v>4.09</v>
       </c>
       <c r="E24" s="6">
         <f t="shared" si="0"/>
-        <v>5.8</v>
+        <v>4.09</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="3" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="H24" s="5"/>
     </row>
-    <row r="25" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>110</v>
+        <v>64</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="C25" s="2">
         <v>1</v>
       </c>
       <c r="D25" s="6">
-        <v>1.46</v>
+        <v>147.52000000000001</v>
       </c>
       <c r="E25" s="6">
         <f t="shared" si="0"/>
-        <v>1.46</v>
+        <v>147.52000000000001</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="3" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="H25" s="5"/>
     </row>
-    <row r="26" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C26" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D26" s="6">
-        <v>2195</v>
+        <v>1.45</v>
       </c>
       <c r="E26" s="6">
         <f t="shared" si="0"/>
-        <v>2195</v>
+        <v>5.8</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="H26" s="5"/>
+    </row>
+    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>77</v>
+        <v>110</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C27" s="2">
         <v>1</v>
       </c>
       <c r="D27" s="6">
-        <v>99.89</v>
+        <v>1.46</v>
       </c>
       <c r="E27" s="6">
         <f t="shared" si="0"/>
-        <v>99.89</v>
+        <v>1.46</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="3" t="s">
-        <v>103</v>
+        <v>72</v>
       </c>
       <c r="H27" s="5"/>
     </row>
-    <row r="28" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C28" s="2">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D28" s="6">
-        <v>6.92</v>
+        <v>2195</v>
       </c>
       <c r="E28" s="6">
         <f t="shared" si="0"/>
-        <v>69.2</v>
+        <v>2195</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="H28" s="5"/>
-    </row>
-    <row r="29" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C29" s="2">
-        <v>2</v>
-      </c>
-      <c r="D29" s="7">
-        <v>72.75</v>
+        <v>1</v>
+      </c>
+      <c r="D29" s="6">
+        <v>99.89</v>
       </c>
       <c r="E29" s="6">
         <f t="shared" si="0"/>
-        <v>145.5</v>
+        <v>99.89</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="3" t="s">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="H29" s="5"/>
     </row>
-    <row r="30" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>101</v>
+        <v>79</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>80</v>
       </c>
       <c r="C30" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D30" s="6">
-        <v>41.17</v>
+        <v>6.92</v>
       </c>
       <c r="E30" s="6">
         <f t="shared" si="0"/>
-        <v>41.17</v>
+        <v>69.2</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>81</v>
+      </c>
+      <c r="H30" s="5"/>
+    </row>
+    <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="C31" s="2">
         <v>2</v>
       </c>
-      <c r="D31" s="6">
-        <v>1.1499999999999999</v>
+      <c r="D31" s="7">
+        <v>72.75</v>
       </c>
       <c r="E31" s="6">
         <f t="shared" si="0"/>
-        <v>2.2999999999999998</v>
+        <v>145.5</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="3" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="H31" s="5"/>
     </row>
-    <row r="32" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>101</v>
       </c>
       <c r="C32" s="2">
         <v>1</v>
       </c>
       <c r="D32" s="6">
-        <v>14.65</v>
+        <v>41.17</v>
       </c>
       <c r="E32" s="6">
         <f t="shared" si="0"/>
-        <v>14.65</v>
+        <v>41.17</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="H32" s="3"/>
-      <c r="I32" s="5"/>
-    </row>
-    <row r="33" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>85</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>117</v>
+        <v>89</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="C33" s="2">
         <v>2</v>
       </c>
-      <c r="D33" s="2">
-        <v>9.85</v>
-      </c>
-      <c r="E33" s="2">
-        <f>C33*D33</f>
-        <v>19.7</v>
-      </c>
-      <c r="F33" s="2"/>
-      <c r="G33" s="8" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D33" s="6">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="E33" s="6">
+        <f t="shared" si="0"/>
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="F33" s="6"/>
+      <c r="G33" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="H33" s="5"/>
+    </row>
+    <row r="34" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C34" s="2">
         <v>1</v>
       </c>
       <c r="D34" s="6">
-        <v>19.989999999999998</v>
+        <v>14.65</v>
       </c>
       <c r="E34" s="6">
         <f t="shared" si="0"/>
-        <v>19.989999999999998</v>
+        <v>14.65</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="H34" s="5"/>
-    </row>
-    <row r="35" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>92</v>
+      </c>
+      <c r="H34" s="3"/>
+      <c r="I34" s="5"/>
+    </row>
+    <row r="35" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>105</v>
+        <v>117</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>118</v>
       </c>
       <c r="C35" s="2">
-        <v>1</v>
-      </c>
-      <c r="D35" s="6">
-        <v>1.87</v>
-      </c>
-      <c r="E35" s="6">
-        <f t="shared" si="0"/>
-        <v>1.87</v>
-      </c>
-      <c r="F35" s="6"/>
-      <c r="G35" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="H35" s="5"/>
-    </row>
-    <row r="36" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+      <c r="D35" s="2">
+        <v>9.85</v>
+      </c>
+      <c r="E35" s="2">
+        <f>C35*D35</f>
+        <v>19.7</v>
+      </c>
+      <c r="F35" s="2"/>
+      <c r="G35" s="8" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C36" s="2">
         <v>1</v>
       </c>
       <c r="D36" s="6">
-        <v>22.56</v>
+        <v>19.989999999999998</v>
       </c>
       <c r="E36" s="6">
         <f t="shared" si="0"/>
-        <v>22.56</v>
+        <v>19.989999999999998</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="3" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="H36" s="5"/>
     </row>
-    <row r="37" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>120</v>
+        <v>106</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>105</v>
       </c>
       <c r="C37" s="2">
-        <v>2</v>
-      </c>
-      <c r="D37" s="2">
-        <v>2.1</v>
+        <v>1</v>
+      </c>
+      <c r="D37" s="6">
+        <v>1.87</v>
       </c>
       <c r="E37" s="6">
         <f t="shared" si="0"/>
-        <v>4.2</v>
+        <v>1.87</v>
       </c>
       <c r="F37" s="6"/>
       <c r="G37" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="H37" s="5"/>
+    </row>
+    <row r="38" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C38" s="2">
+        <v>1</v>
+      </c>
+      <c r="D38" s="6">
+        <v>22.56</v>
+      </c>
+      <c r="E38" s="6">
+        <f t="shared" si="0"/>
+        <v>22.56</v>
+      </c>
+      <c r="F38" s="6"/>
+      <c r="G38" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="H38" s="5"/>
+    </row>
+    <row r="39" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C39" s="2">
+        <v>2</v>
+      </c>
+      <c r="D39" s="2">
+        <v>2.1</v>
+      </c>
+      <c r="E39" s="6">
+        <f t="shared" si="0"/>
+        <v>4.2</v>
+      </c>
+      <c r="F39" s="6"/>
+      <c r="G39" s="3" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A38" s="2" t="s">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B40" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C38" s="2">
+      <c r="C40" s="2">
         <v>4</v>
       </c>
-      <c r="D38" s="6">
+      <c r="D40" s="6">
         <v>3.75</v>
       </c>
-      <c r="E38" s="6">
+      <c r="E40" s="6">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="F38" s="6"/>
-      <c r="G38" s="1" t="s">
+      <c r="F40" s="6"/>
+      <c r="G40" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A39" s="2" t="s">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B41" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="C39" s="2">
-        <v>1</v>
-      </c>
-      <c r="D39" s="2">
+      <c r="C41" s="2">
+        <v>1</v>
+      </c>
+      <c r="D41" s="2">
         <v>299.54000000000002</v>
       </c>
-      <c r="E39" s="2">
+      <c r="E41" s="2">
         <f t="shared" si="0"/>
         <v>299.54000000000002</v>
       </c>
-      <c r="F39" s="2"/>
-      <c r="G39" s="8" t="s">
+      <c r="F41" s="2"/>
+      <c r="G41" s="8" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A40" s="2" t="s">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B42" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C40" s="2">
+      <c r="C42" s="2">
         <v>2</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D42" s="2">
         <v>6.74</v>
       </c>
-      <c r="E40" s="2">
+      <c r="E42" s="2">
         <f t="shared" si="0"/>
         <v>13.48</v>
       </c>
-      <c r="F40" s="2" t="s">
+      <c r="F42" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="G40" s="1" t="s">
+      <c r="G42" s="1" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A41" s="2" t="s">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B43" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="C41" s="2">
-        <v>1</v>
-      </c>
-      <c r="D41" s="2">
+      <c r="C43" s="2">
+        <v>1</v>
+      </c>
+      <c r="D43" s="2">
         <v>15.89</v>
       </c>
-      <c r="E41">
+      <c r="E43">
         <v>15.89</v>
       </c>
-      <c r="G41" s="1" t="s">
+      <c r="G43" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A42" s="2" t="s">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B44" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="C42" s="2">
+      <c r="C44" s="2">
         <v>4</v>
       </c>
-      <c r="D42" s="7">
+      <c r="D44" s="7">
         <v>2.0699999999999998</v>
       </c>
-      <c r="E42" s="6">
+      <c r="E44" s="6">
         <v>12.41</v>
       </c>
-      <c r="F42" s="6" t="s">
+      <c r="F44" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="G42" s="1" t="s">
+      <c r="G44" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="H42" s="1" t="s">
+      <c r="H44" s="1" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A43" s="2" t="s">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B45" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="C43" s="2">
-        <v>1</v>
-      </c>
-      <c r="D43" s="7">
+      <c r="C45" s="2">
+        <v>1</v>
+      </c>
+      <c r="D45" s="7">
         <v>4.3600000000000003</v>
       </c>
-      <c r="E43" s="7">
+      <c r="E45" s="7">
         <v>4.3600000000000003</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="H43" s="1"/>
-    </row>
-    <row r="44" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A44" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="B44" s="10" t="s">
-        <v>153</v>
-      </c>
-      <c r="C44" s="2">
-        <v>1</v>
-      </c>
-      <c r="D44" s="7">
-        <v>2.73</v>
-      </c>
-      <c r="E44" s="6">
-        <v>2.73</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="G44" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="H44" s="1"/>
-    </row>
-    <row r="45" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A45" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="B45" s="9" t="s">
-        <v>152</v>
-      </c>
-      <c r="C45" s="2">
-        <v>1</v>
-      </c>
-      <c r="D45" s="7">
-        <v>1.2</v>
-      </c>
-      <c r="E45" s="6">
-        <v>1.2</v>
       </c>
       <c r="F45" s="6" t="s">
         <v>147</v>
       </c>
       <c r="G45" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="H45" s="1"/>
+    </row>
+    <row r="46" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A46" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B46" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="C46" s="2">
+        <v>1</v>
+      </c>
+      <c r="D46" s="7">
+        <v>2.73</v>
+      </c>
+      <c r="E46" s="6">
+        <v>2.73</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="H46" s="1"/>
+    </row>
+    <row r="47" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A47" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="C47" s="2">
+        <v>1</v>
+      </c>
+      <c r="D47" s="7">
+        <v>1.2</v>
+      </c>
+      <c r="E47" s="6">
+        <v>1.2</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="G47" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="H45" s="1"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="7"/>
-      <c r="E46" s="6"/>
-      <c r="F46" s="6"/>
-      <c r="G46" s="1"/>
-      <c r="H46" s="1"/>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="6"/>
-      <c r="F47" s="6"/>
-      <c r="G47" s="1"/>
       <c r="H47" s="1"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D48" s="7" t="s">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="6"/>
+      <c r="F48" s="6"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A49" s="2"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="7"/>
+      <c r="E49" s="6"/>
+      <c r="F49" s="6"/>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D50" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E48" s="6">
-        <f>SUM(E3:E42)</f>
-        <v>12767.039999999995</v>
+      <c r="E50" s="6">
+        <f>SUM(E3:E44)</f>
+        <v>12788.479999999994</v>
       </c>
     </row>
   </sheetData>
@@ -2047,42 +2128,42 @@
     <hyperlink ref="G8" r:id="rId5" xr:uid="{BE59E38F-DA22-4ED1-BF36-E84DE0018044}"/>
     <hyperlink ref="G7" r:id="rId6" xr:uid="{843281D0-FA21-4F36-A652-0F07141A7B84}"/>
     <hyperlink ref="G3" r:id="rId7" xr:uid="{AC5FA834-82E0-404E-B150-C4F68DA38C6A}"/>
-    <hyperlink ref="G9" r:id="rId8" xr:uid="{30A401D7-C620-43B9-9D9E-19B3DC7BF553}"/>
-    <hyperlink ref="G10" r:id="rId9" xr:uid="{9E7C13BC-99F6-4C00-8247-D65DF4039E02}"/>
-    <hyperlink ref="G12" r:id="rId10" xr:uid="{D9870AF0-1C4B-473B-8416-474E754D5E7E}"/>
-    <hyperlink ref="G13" r:id="rId11" xr:uid="{7E2805CC-0B04-4DB0-9F38-3741F75A7D1D}"/>
-    <hyperlink ref="G14" r:id="rId12" xr:uid="{6AF56708-0BAB-42E8-A3AE-FD431334CF6C}"/>
-    <hyperlink ref="G15" r:id="rId13" xr:uid="{F2324ACB-C085-42C4-8640-3C360A4D119E}"/>
-    <hyperlink ref="G18" r:id="rId14" xr:uid="{36F5D6E3-807C-49A7-8D30-80566D9949D4}"/>
-    <hyperlink ref="G20" r:id="rId15" xr:uid="{1F94BCB9-4D2C-4C92-8BF0-A4FC479E37E8}"/>
-    <hyperlink ref="G21" r:id="rId16" xr:uid="{6624F982-B428-4251-AA28-31179DCD8937}"/>
-    <hyperlink ref="G22" r:id="rId17" xr:uid="{58E2A489-0714-4655-8748-622D874EF6F8}"/>
-    <hyperlink ref="G23" r:id="rId18" xr:uid="{81E87505-E60E-4515-89EA-9361938F7388}"/>
-    <hyperlink ref="G24" r:id="rId19" xr:uid="{EFDA772F-CC83-4998-A756-1FADE307C734}"/>
-    <hyperlink ref="G25" r:id="rId20" xr:uid="{F81462CE-4E7C-4FAB-8A8E-D305901B6FCF}"/>
-    <hyperlink ref="G28" r:id="rId21" xr:uid="{0B3AB74B-6B3E-4207-9645-7AB7D6617AD3}"/>
-    <hyperlink ref="G29" r:id="rId22" xr:uid="{5CF86D47-7D87-4635-9306-B8490C771687}"/>
-    <hyperlink ref="G30" r:id="rId23" display="https://www.digikey.com/en/products/detail/belden-inc/35618-002500/7041945?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=22518541616&amp;gbraid=0AAAAADrbLljEBpjA6o11517XtnCbKLnsR&amp;gclid=Cj0KCQjwuKnGBhD5ARIsAD19Rsa4nb1dzOV49q-F9Xe7dRzLg9fr09jgomA5Q7py5DmHjVBe4NA0heoaAspGEALw_wcB" xr:uid="{A2DDC80C-6F39-4C44-B776-452B7FA8CAC3}"/>
-    <hyperlink ref="G31" r:id="rId24" xr:uid="{71E7E2F7-3EA3-469E-BDBD-A5E1E2E4F347}"/>
-    <hyperlink ref="G32" r:id="rId25" xr:uid="{F2165E25-79D9-4521-9261-0FF86CB8CEB1}"/>
-    <hyperlink ref="G11" r:id="rId26" xr:uid="{2459F536-6BF7-4F95-8ED6-65EBE68E0306}"/>
+    <hyperlink ref="G11" r:id="rId8" xr:uid="{30A401D7-C620-43B9-9D9E-19B3DC7BF553}"/>
+    <hyperlink ref="G12" r:id="rId9" xr:uid="{9E7C13BC-99F6-4C00-8247-D65DF4039E02}"/>
+    <hyperlink ref="G14" r:id="rId10" xr:uid="{D9870AF0-1C4B-473B-8416-474E754D5E7E}"/>
+    <hyperlink ref="G15" r:id="rId11" xr:uid="{7E2805CC-0B04-4DB0-9F38-3741F75A7D1D}"/>
+    <hyperlink ref="G16" r:id="rId12" xr:uid="{6AF56708-0BAB-42E8-A3AE-FD431334CF6C}"/>
+    <hyperlink ref="G17" r:id="rId13" xr:uid="{F2324ACB-C085-42C4-8640-3C360A4D119E}"/>
+    <hyperlink ref="G20" r:id="rId14" xr:uid="{36F5D6E3-807C-49A7-8D30-80566D9949D4}"/>
+    <hyperlink ref="G22" r:id="rId15" xr:uid="{1F94BCB9-4D2C-4C92-8BF0-A4FC479E37E8}"/>
+    <hyperlink ref="G23" r:id="rId16" xr:uid="{6624F982-B428-4251-AA28-31179DCD8937}"/>
+    <hyperlink ref="G24" r:id="rId17" xr:uid="{58E2A489-0714-4655-8748-622D874EF6F8}"/>
+    <hyperlink ref="G25" r:id="rId18" xr:uid="{81E87505-E60E-4515-89EA-9361938F7388}"/>
+    <hyperlink ref="G26" r:id="rId19" xr:uid="{EFDA772F-CC83-4998-A756-1FADE307C734}"/>
+    <hyperlink ref="G27" r:id="rId20" xr:uid="{F81462CE-4E7C-4FAB-8A8E-D305901B6FCF}"/>
+    <hyperlink ref="G30" r:id="rId21" xr:uid="{0B3AB74B-6B3E-4207-9645-7AB7D6617AD3}"/>
+    <hyperlink ref="G31" r:id="rId22" xr:uid="{5CF86D47-7D87-4635-9306-B8490C771687}"/>
+    <hyperlink ref="G32" r:id="rId23" display="https://www.digikey.com/en/products/detail/belden-inc/35618-002500/7041945?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=22518541616&amp;gbraid=0AAAAADrbLljEBpjA6o11517XtnCbKLnsR&amp;gclid=Cj0KCQjwuKnGBhD5ARIsAD19Rsa4nb1dzOV49q-F9Xe7dRzLg9fr09jgomA5Q7py5DmHjVBe4NA0heoaAspGEALw_wcB" xr:uid="{A2DDC80C-6F39-4C44-B776-452B7FA8CAC3}"/>
+    <hyperlink ref="G33" r:id="rId24" xr:uid="{71E7E2F7-3EA3-469E-BDBD-A5E1E2E4F347}"/>
+    <hyperlink ref="G34" r:id="rId25" xr:uid="{F2165E25-79D9-4521-9261-0FF86CB8CEB1}"/>
+    <hyperlink ref="G13" r:id="rId26" xr:uid="{2459F536-6BF7-4F95-8ED6-65EBE68E0306}"/>
     <hyperlink ref="H6" r:id="rId27" xr:uid="{A8C35020-1C53-4073-BE6C-0F6933CB1921}"/>
     <hyperlink ref="H5" r:id="rId28" xr:uid="{A49999D0-0D24-4148-A259-6949303F3996}"/>
     <hyperlink ref="H7" r:id="rId29" xr:uid="{D90F92BC-9947-4813-8C28-6009DA178051}"/>
-    <hyperlink ref="G26" r:id="rId30" xr:uid="{F3415021-EB69-4CB6-B212-558D2454FF2B}"/>
-    <hyperlink ref="H26" r:id="rId31" xr:uid="{E4EF5DF5-36DD-4B50-AF25-A19F9CE4857A}"/>
-    <hyperlink ref="H30" r:id="rId32" xr:uid="{5A940B12-DD8E-47F3-8C44-FCBBD353757C}"/>
-    <hyperlink ref="G35" r:id="rId33" display="https://www.digikey.com/en/products/detail/io-audio-technologies/IO-C14SP-63/21379594?gad_source=1&amp;gad_campaignid=22396809060&amp;gbraid=0AAAAADrbLlisC8UtMjpExL2rbCWoG3ieR&amp;gclid=Cj0KCQjw0NPGBhCDARIsAGAzpp2VLlJaqhBiZUHDGRJcszbohHTDT2yecNaX-w7lJU8lPrGXw1UWNiwaAsExEALw_wcB&amp;gclsrc=aw.ds" xr:uid="{4B8089ED-EC5B-48CB-8DCC-6C3B9EB37FA7}"/>
-    <hyperlink ref="G36" r:id="rId34" xr:uid="{E263962D-47C1-49F9-A559-36360176D757}"/>
-    <hyperlink ref="G16" r:id="rId35" xr:uid="{83A27BB2-9C4A-4120-9925-FBAA61079743}"/>
-    <hyperlink ref="G33" r:id="rId36" xr:uid="{1E1A9060-9FD1-40EB-9CB4-035E777CB97F}"/>
-    <hyperlink ref="G17" r:id="rId37" xr:uid="{E3301FAD-92C1-4805-8EF6-30AE4F47746A}"/>
-    <hyperlink ref="G38" r:id="rId38" xr:uid="{94087BF9-485B-4DE1-AA9E-568F4259E676}"/>
-    <hyperlink ref="G40" r:id="rId39" xr:uid="{6D79D5B6-03CD-4FCF-94AD-8DF566E11950}"/>
-    <hyperlink ref="G41" r:id="rId40" display="https://nam02.safelinks.protection.outlook.com/?url=https%3A%2F%2Fwww.grainger.com%2Fproduct%2FMILWAUKEE-Hole-Saw-1-in-Saw-Dia-856EV8&amp;data=05%7C02%7CCKB11%40email.sc.edu%7C9a1df447a7c2434dc85d08de157fc0b4%7C4b2a4b19d135420e8bb2b1cd238998cc%7C0%7C0%7C638971835598967940%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=EAjn5hwuV%2BewMqz9WyyZN%2Fqwh4VRByeEbQ3Le73uExc%3D&amp;reserved=0" xr:uid="{A9796287-2762-473D-888E-E0F37F2D5222}"/>
-    <hyperlink ref="H42" r:id="rId41" xr:uid="{B771626B-BE96-4E86-B8E7-5F4D421B11CC}"/>
-    <hyperlink ref="G27" r:id="rId42" xr:uid="{9087F97E-6A29-4916-9C63-C220AC3B6655}"/>
-    <hyperlink ref="G37" r:id="rId43" xr:uid="{3FA6174D-CFA4-4F51-8AB7-928DB84B83AE}"/>
+    <hyperlink ref="G28" r:id="rId30" xr:uid="{F3415021-EB69-4CB6-B212-558D2454FF2B}"/>
+    <hyperlink ref="H28" r:id="rId31" xr:uid="{E4EF5DF5-36DD-4B50-AF25-A19F9CE4857A}"/>
+    <hyperlink ref="H32" r:id="rId32" xr:uid="{5A940B12-DD8E-47F3-8C44-FCBBD353757C}"/>
+    <hyperlink ref="G37" r:id="rId33" display="https://www.digikey.com/en/products/detail/io-audio-technologies/IO-C14SP-63/21379594?gad_source=1&amp;gad_campaignid=22396809060&amp;gbraid=0AAAAADrbLlisC8UtMjpExL2rbCWoG3ieR&amp;gclid=Cj0KCQjw0NPGBhCDARIsAGAzpp2VLlJaqhBiZUHDGRJcszbohHTDT2yecNaX-w7lJU8lPrGXw1UWNiwaAsExEALw_wcB&amp;gclsrc=aw.ds" xr:uid="{4B8089ED-EC5B-48CB-8DCC-6C3B9EB37FA7}"/>
+    <hyperlink ref="G38" r:id="rId34" xr:uid="{E263962D-47C1-49F9-A559-36360176D757}"/>
+    <hyperlink ref="G18" r:id="rId35" xr:uid="{83A27BB2-9C4A-4120-9925-FBAA61079743}"/>
+    <hyperlink ref="G35" r:id="rId36" xr:uid="{1E1A9060-9FD1-40EB-9CB4-035E777CB97F}"/>
+    <hyperlink ref="G19" r:id="rId37" xr:uid="{E3301FAD-92C1-4805-8EF6-30AE4F47746A}"/>
+    <hyperlink ref="G40" r:id="rId38" xr:uid="{94087BF9-485B-4DE1-AA9E-568F4259E676}"/>
+    <hyperlink ref="G42" r:id="rId39" xr:uid="{6D79D5B6-03CD-4FCF-94AD-8DF566E11950}"/>
+    <hyperlink ref="G43" r:id="rId40" display="https://nam02.safelinks.protection.outlook.com/?url=https%3A%2F%2Fwww.grainger.com%2Fproduct%2FMILWAUKEE-Hole-Saw-1-in-Saw-Dia-856EV8&amp;data=05%7C02%7CCKB11%40email.sc.edu%7C9a1df447a7c2434dc85d08de157fc0b4%7C4b2a4b19d135420e8bb2b1cd238998cc%7C0%7C0%7C638971835598967940%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=EAjn5hwuV%2BewMqz9WyyZN%2Fqwh4VRByeEbQ3Le73uExc%3D&amp;reserved=0" xr:uid="{A9796287-2762-473D-888E-E0F37F2D5222}"/>
+    <hyperlink ref="H44" r:id="rId41" xr:uid="{B771626B-BE96-4E86-B8E7-5F4D421B11CC}"/>
+    <hyperlink ref="G29" r:id="rId42" xr:uid="{9087F97E-6A29-4916-9C63-C220AC3B6655}"/>
+    <hyperlink ref="G39" r:id="rId43" xr:uid="{3FA6174D-CFA4-4F51-8AB7-928DB84B83AE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId44"/>

</xml_diff>